<commit_message>
fix: sanitize publication text and metadata with verified original archives
</commit_message>
<xml_diff>
--- a/docs/go2-produktionsreihenfolge/source/woek_go2_produktionsreihenfolge_detailkonzepte_v1_0.xlsx
+++ b/docs/go2-produktionsreihenfolge/source/woek_go2_produktionsreihenfolge_detailkonzepte_v1_0.xlsx
@@ -257,9 +257,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Wirkungsoekonomie">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Wirkungsoekonomie">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -309,7 +309,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Wirkungsoekonomie">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -414,7 +414,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Go 2 – Produktionsreihenfolge echte Detailkonzepte</x:v>
+        <x:v>Go 2 - Produktionsreihenfolge echte Detailkonzepte</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str"/>
       <x:c r="C1" s="5" t="str"/>

</xml_diff>

<commit_message>
chore: Oracle Wirkungsticker wake-up 2026-09-06T14:50:09Z
</commit_message>
<xml_diff>
--- a/docs/go2-produktionsreihenfolge/source/woek_go2_produktionsreihenfolge_detailkonzepte_v1_0.xlsx
+++ b/docs/go2-produktionsreihenfolge/source/woek_go2_produktionsreihenfolge_detailkonzepte_v1_0.xlsx
@@ -257,9 +257,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Wirkungsoekonomie">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Wirkungsoekonomie">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -309,7 +309,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Wirkungsoekonomie">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -414,7 +414,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Go 2 – Produktionsreihenfolge echte Detailkonzepte</x:v>
+        <x:v>Go 2 - Produktionsreihenfolge echte Detailkonzepte</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str"/>
       <x:c r="C1" s="5" t="str"/>

</xml_diff>

<commit_message>
chore: Oracle Wirkungsticker wake-up 2026-09-06T18:05:27Z
</commit_message>
<xml_diff>
--- a/docs/go2-produktionsreihenfolge/source/woek_go2_produktionsreihenfolge_detailkonzepte_v1_0.xlsx
+++ b/docs/go2-produktionsreihenfolge/source/woek_go2_produktionsreihenfolge_detailkonzepte_v1_0.xlsx
@@ -257,9 +257,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Wirkungsoekonomie">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Wirkungsoekonomie">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -309,7 +309,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Wirkungsoekonomie">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -414,7 +414,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>Go 2 – Produktionsreihenfolge echte Detailkonzepte</x:v>
+        <x:v>Go 2 - Produktionsreihenfolge echte Detailkonzepte</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str"/>
       <x:c r="C1" s="5" t="str"/>

</xml_diff>